<commit_message>
add: update W05 assessment and challenge files
</commit_message>
<xml_diff>
--- a/01-essentials/material_curso/modulo-05/W05-Assessment.xlsx
+++ b/01-essentials/material_curso/modulo-05/W05-Assessment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Proyectos\ExcelLearning\01-essentials\material_curso\modulo-05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA3AE29-67B9-418C-9FB1-8A3DEF8A95A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E766071-69B2-4655-9893-0BEBAFAAE7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="83">
   <si>
     <t>Student No</t>
   </si>
@@ -290,9 +290,6 @@
   </si>
   <si>
     <t>Ms Simpson</t>
-  </si>
-  <si>
-    <t>sss</t>
   </si>
 </sst>
 </file>
@@ -830,9 +827,7 @@
       <c r="C4" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>83</v>
-      </c>
+      <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
         <v>73</v>
       </c>

</xml_diff>